<commit_message>
Ethiopia: Month 1 = Oct 2026
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_014bhqta51kFyf2UMB6E5eD3
</commit_message>
<xml_diff>
--- a/out/Milestone_Valid_Months.xlsx
+++ b/out/Milestone_Valid_Months.xlsx
@@ -3687,17 +3687,17 @@
       </c>
       <c r="C62" t="inlineStr">
         <is>
-          <t>Sep-26 to Feb-27</t>
+          <t>Oct-26 to Mar-27</t>
         </is>
       </c>
       <c r="D62" t="inlineStr">
         <is>
-          <t>Sep-26</t>
+          <t>Oct-26</t>
         </is>
       </c>
       <c r="E62" t="inlineStr">
         <is>
-          <t>Feb-27</t>
+          <t>Mar-27</t>
         </is>
       </c>
       <c r="F62" t="n">
@@ -3715,12 +3715,12 @@
       </c>
       <c r="I62" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>High</t>
         </is>
       </c>
       <c r="J62" s="1" t="inlineStr">
         <is>
-          <t>ASSUMED: no calendar anchor in file; Sep-26 assumed (same template family / Sept 21 2026 start)</t>
+          <t>Month 1 = Oct-26 per user (file itself has no calendar anchor)</t>
         </is>
       </c>
       <c r="K62" t="inlineStr">
@@ -3742,17 +3742,17 @@
       </c>
       <c r="C63" t="inlineStr">
         <is>
-          <t>Sep-26 to Feb-27</t>
+          <t>Oct-26 to Mar-27</t>
         </is>
       </c>
       <c r="D63" t="inlineStr">
         <is>
-          <t>Sep-26</t>
+          <t>Oct-26</t>
         </is>
       </c>
       <c r="E63" t="inlineStr">
         <is>
-          <t>Feb-27</t>
+          <t>Mar-27</t>
         </is>
       </c>
       <c r="F63" t="n">
@@ -3770,12 +3770,12 @@
       </c>
       <c r="I63" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>High</t>
         </is>
       </c>
       <c r="J63" s="1" t="inlineStr">
         <is>
-          <t>ASSUMED: no calendar anchor in file; Sep-26 assumed (same template family / Sept 21 2026 start)</t>
+          <t>Month 1 = Oct-26 per user (file itself has no calendar anchor)</t>
         </is>
       </c>
       <c r="K63" t="inlineStr">
@@ -3797,17 +3797,17 @@
       </c>
       <c r="C64" t="inlineStr">
         <is>
-          <t>Sep-26 to Feb-27</t>
+          <t>Oct-26 to Mar-27</t>
         </is>
       </c>
       <c r="D64" t="inlineStr">
         <is>
-          <t>Sep-26</t>
+          <t>Oct-26</t>
         </is>
       </c>
       <c r="E64" t="inlineStr">
         <is>
-          <t>Feb-27</t>
+          <t>Mar-27</t>
         </is>
       </c>
       <c r="F64" t="n">
@@ -3825,12 +3825,12 @@
       </c>
       <c r="I64" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>High</t>
         </is>
       </c>
       <c r="J64" s="1" t="inlineStr">
         <is>
-          <t>ASSUMED: no calendar anchor in file; Sep-26 assumed (same template family / Sept 21 2026 start)</t>
+          <t>Month 1 = Oct-26 per user (file itself has no calendar anchor)</t>
         </is>
       </c>
       <c r="K64" t="inlineStr">
@@ -3852,17 +3852,17 @@
       </c>
       <c r="C65" t="inlineStr">
         <is>
-          <t>Sep-26 to Feb-27</t>
+          <t>Oct-26 to Mar-27</t>
         </is>
       </c>
       <c r="D65" t="inlineStr">
         <is>
-          <t>Sep-26</t>
+          <t>Oct-26</t>
         </is>
       </c>
       <c r="E65" t="inlineStr">
         <is>
-          <t>Feb-27</t>
+          <t>Mar-27</t>
         </is>
       </c>
       <c r="F65" t="n">
@@ -3880,12 +3880,12 @@
       </c>
       <c r="I65" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>High</t>
         </is>
       </c>
       <c r="J65" s="1" t="inlineStr">
         <is>
-          <t>ASSUMED: no calendar anchor in file; Sep-26 assumed (same template family / Sept 21 2026 start)</t>
+          <t>Month 1 = Oct-26 per user (file itself has no calendar anchor)</t>
         </is>
       </c>
       <c r="K65" t="inlineStr">
@@ -3907,17 +3907,17 @@
       </c>
       <c r="C66" t="inlineStr">
         <is>
-          <t>Oct-26 to Mar-27</t>
+          <t>Nov-26 to Apr-27</t>
         </is>
       </c>
       <c r="D66" t="inlineStr">
         <is>
-          <t>Oct-26</t>
+          <t>Nov-26</t>
         </is>
       </c>
       <c r="E66" t="inlineStr">
         <is>
-          <t>Mar-27</t>
+          <t>Apr-27</t>
         </is>
       </c>
       <c r="F66" t="n">
@@ -3935,12 +3935,12 @@
       </c>
       <c r="I66" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>High</t>
         </is>
       </c>
       <c r="J66" s="1" t="inlineStr">
         <is>
-          <t>ASSUMED: no calendar anchor in file; Sep-26 assumed (same template family / Sept 21 2026 start)</t>
+          <t>Month 1 = Oct-26 per user (file itself has no calendar anchor)</t>
         </is>
       </c>
       <c r="K66" t="inlineStr">
@@ -3962,17 +3962,17 @@
       </c>
       <c r="C67" t="inlineStr">
         <is>
-          <t>Oct-26 to Mar-27</t>
+          <t>Nov-26 to Apr-27</t>
         </is>
       </c>
       <c r="D67" t="inlineStr">
         <is>
-          <t>Oct-26</t>
+          <t>Nov-26</t>
         </is>
       </c>
       <c r="E67" t="inlineStr">
         <is>
-          <t>Mar-27</t>
+          <t>Apr-27</t>
         </is>
       </c>
       <c r="F67" t="n">
@@ -3990,12 +3990,12 @@
       </c>
       <c r="I67" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>High</t>
         </is>
       </c>
       <c r="J67" s="1" t="inlineStr">
         <is>
-          <t>ASSUMED: no calendar anchor in file; Sep-26 assumed (same template family / Sept 21 2026 start)</t>
+          <t>Month 1 = Oct-26 per user (file itself has no calendar anchor)</t>
         </is>
       </c>
       <c r="K67" t="inlineStr">
@@ -4017,17 +4017,17 @@
       </c>
       <c r="C68" t="inlineStr">
         <is>
-          <t>Oct-26 to May-27</t>
+          <t>Nov-26 to Jun-27</t>
         </is>
       </c>
       <c r="D68" t="inlineStr">
         <is>
-          <t>Oct-26</t>
+          <t>Nov-26</t>
         </is>
       </c>
       <c r="E68" t="inlineStr">
         <is>
-          <t>May-27</t>
+          <t>Jun-27</t>
         </is>
       </c>
       <c r="F68" t="n">
@@ -4045,12 +4045,12 @@
       </c>
       <c r="I68" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>High</t>
         </is>
       </c>
       <c r="J68" s="1" t="inlineStr">
         <is>
-          <t>ASSUMED: no calendar anchor in file; Sep-26 assumed (same template family / Sept 21 2026 start)</t>
+          <t>Month 1 = Oct-26 per user (file itself has no calendar anchor)</t>
         </is>
       </c>
       <c r="K68" t="inlineStr">
@@ -4072,17 +4072,17 @@
       </c>
       <c r="C69" t="inlineStr">
         <is>
-          <t>Nov-26 to May-27</t>
+          <t>Dec-26 to Jun-27</t>
         </is>
       </c>
       <c r="D69" t="inlineStr">
         <is>
-          <t>Nov-26</t>
+          <t>Dec-26</t>
         </is>
       </c>
       <c r="E69" t="inlineStr">
         <is>
-          <t>May-27</t>
+          <t>Jun-27</t>
         </is>
       </c>
       <c r="F69" t="n">
@@ -4100,12 +4100,12 @@
       </c>
       <c r="I69" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>High</t>
         </is>
       </c>
       <c r="J69" s="1" t="inlineStr">
         <is>
-          <t>ASSUMED: no calendar anchor in file; Sep-26 assumed (same template family / Sept 21 2026 start)</t>
+          <t>Month 1 = Oct-26 per user (file itself has no calendar anchor)</t>
         </is>
       </c>
       <c r="K69" t="inlineStr">
@@ -4127,17 +4127,17 @@
       </c>
       <c r="C70" t="inlineStr">
         <is>
-          <t>Nov-26 to Aug-27</t>
+          <t>Dec-26 to Sep-27</t>
         </is>
       </c>
       <c r="D70" t="inlineStr">
         <is>
-          <t>Nov-26</t>
+          <t>Dec-26</t>
         </is>
       </c>
       <c r="E70" t="inlineStr">
         <is>
-          <t>Aug-27</t>
+          <t>Sep-27</t>
         </is>
       </c>
       <c r="F70" t="n">
@@ -4155,12 +4155,12 @@
       </c>
       <c r="I70" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>High</t>
         </is>
       </c>
       <c r="J70" s="1" t="inlineStr">
         <is>
-          <t>ASSUMED: no calendar anchor in file; Sep-26 assumed (same template family / Sept 21 2026 start)</t>
+          <t>Month 1 = Oct-26 per user (file itself has no calendar anchor)</t>
         </is>
       </c>
       <c r="K70" t="inlineStr">
@@ -4182,17 +4182,17 @@
       </c>
       <c r="C71" t="inlineStr">
         <is>
-          <t>Sep-26 to Feb-27</t>
+          <t>Oct-26 to Mar-27</t>
         </is>
       </c>
       <c r="D71" t="inlineStr">
         <is>
-          <t>Sep-26</t>
+          <t>Oct-26</t>
         </is>
       </c>
       <c r="E71" t="inlineStr">
         <is>
-          <t>Feb-27</t>
+          <t>Mar-27</t>
         </is>
       </c>
       <c r="F71" t="n">
@@ -4210,12 +4210,12 @@
       </c>
       <c r="I71" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>High</t>
         </is>
       </c>
       <c r="J71" s="1" t="inlineStr">
         <is>
-          <t>ASSUMED: no calendar anchor in file; Sep-26 assumed (same template family / Sept 21 2026 start)</t>
+          <t>Month 1 = Oct-26 per user (file itself has no calendar anchor)</t>
         </is>
       </c>
       <c r="K71" t="inlineStr">
@@ -4237,17 +4237,17 @@
       </c>
       <c r="C72" t="inlineStr">
         <is>
-          <t>Dec-26 to Jun-27</t>
+          <t>Jan-27 to Jul-27</t>
         </is>
       </c>
       <c r="D72" t="inlineStr">
         <is>
-          <t>Dec-26</t>
+          <t>Jan-27</t>
         </is>
       </c>
       <c r="E72" t="inlineStr">
         <is>
-          <t>Jun-27</t>
+          <t>Jul-27</t>
         </is>
       </c>
       <c r="F72" t="n">
@@ -4265,12 +4265,12 @@
       </c>
       <c r="I72" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>High</t>
         </is>
       </c>
       <c r="J72" s="1" t="inlineStr">
         <is>
-          <t>ASSUMED: no calendar anchor in file; Sep-26 assumed (same template family / Sept 21 2026 start)</t>
+          <t>Month 1 = Oct-26 per user (file itself has no calendar anchor)</t>
         </is>
       </c>
       <c r="K72" t="inlineStr">
@@ -4292,17 +4292,17 @@
       </c>
       <c r="C73" t="inlineStr">
         <is>
-          <t>Dec-26 to Jun-27</t>
+          <t>Jan-27 to Jul-27</t>
         </is>
       </c>
       <c r="D73" t="inlineStr">
         <is>
-          <t>Dec-26</t>
+          <t>Jan-27</t>
         </is>
       </c>
       <c r="E73" t="inlineStr">
         <is>
-          <t>Jun-27</t>
+          <t>Jul-27</t>
         </is>
       </c>
       <c r="F73" t="n">
@@ -4320,12 +4320,12 @@
       </c>
       <c r="I73" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>High</t>
         </is>
       </c>
       <c r="J73" s="1" t="inlineStr">
         <is>
-          <t>ASSUMED: no calendar anchor in file; Sep-26 assumed (same template family / Sept 21 2026 start)</t>
+          <t>Month 1 = Oct-26 per user (file itself has no calendar anchor)</t>
         </is>
       </c>
       <c r="K73" t="inlineStr">
@@ -4347,17 +4347,17 @@
       </c>
       <c r="C74" t="inlineStr">
         <is>
-          <t>Dec-26 to Jun-27</t>
+          <t>Jan-27 to Jul-27</t>
         </is>
       </c>
       <c r="D74" t="inlineStr">
         <is>
-          <t>Dec-26</t>
+          <t>Jan-27</t>
         </is>
       </c>
       <c r="E74" t="inlineStr">
         <is>
-          <t>Jun-27</t>
+          <t>Jul-27</t>
         </is>
       </c>
       <c r="F74" t="n">
@@ -4375,12 +4375,12 @@
       </c>
       <c r="I74" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>High</t>
         </is>
       </c>
       <c r="J74" s="1" t="inlineStr">
         <is>
-          <t>ASSUMED: no calendar anchor in file; Sep-26 assumed (same template family / Sept 21 2026 start)</t>
+          <t>Month 1 = Oct-26 per user (file itself has no calendar anchor)</t>
         </is>
       </c>
       <c r="K74" t="inlineStr">
@@ -4402,17 +4402,17 @@
       </c>
       <c r="C75" t="inlineStr">
         <is>
-          <t>Jan-27 to Aug-27</t>
+          <t>Feb-27 to Sep-27</t>
         </is>
       </c>
       <c r="D75" t="inlineStr">
         <is>
-          <t>Jan-27</t>
+          <t>Feb-27</t>
         </is>
       </c>
       <c r="E75" t="inlineStr">
         <is>
-          <t>Aug-27</t>
+          <t>Sep-27</t>
         </is>
       </c>
       <c r="F75" t="n">
@@ -4430,12 +4430,12 @@
       </c>
       <c r="I75" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>High</t>
         </is>
       </c>
       <c r="J75" s="1" t="inlineStr">
         <is>
-          <t>ASSUMED: no calendar anchor in file; Sep-26 assumed (same template family / Sept 21 2026 start)</t>
+          <t>Month 1 = Oct-26 per user (file itself has no calendar anchor)</t>
         </is>
       </c>
       <c r="K75" t="inlineStr">
@@ -4457,17 +4457,17 @@
       </c>
       <c r="C76" t="inlineStr">
         <is>
-          <t>Sep-26 to Oct-26</t>
+          <t>Oct-26 to Nov-26</t>
         </is>
       </c>
       <c r="D76" t="inlineStr">
         <is>
-          <t>Sep-26</t>
+          <t>Oct-26</t>
         </is>
       </c>
       <c r="E76" t="inlineStr">
         <is>
-          <t>Oct-26</t>
+          <t>Nov-26</t>
         </is>
       </c>
       <c r="F76" t="n">
@@ -4485,12 +4485,12 @@
       </c>
       <c r="I76" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>High</t>
         </is>
       </c>
       <c r="J76" s="1" t="inlineStr">
         <is>
-          <t>ASSUMED: no calendar anchor in file; Sep-26 assumed (same template family / Sept 21 2026 start)</t>
+          <t>Month 1 = Oct-26 per user (file itself has no calendar anchor)</t>
         </is>
       </c>
       <c r="K76" t="inlineStr">
@@ -19642,11 +19642,11 @@
       </c>
       <c r="C387" t="inlineStr">
         <is>
-          <t>Sep-26</t>
+          <t>Oct-26</t>
         </is>
       </c>
       <c r="D387" s="2" t="n">
-        <v>46266</v>
+        <v>46296</v>
       </c>
       <c r="E387" t="inlineStr">
         <is>
@@ -19655,7 +19655,7 @@
       </c>
       <c r="F387" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>High</t>
         </is>
       </c>
     </row>
@@ -19672,11 +19672,11 @@
       </c>
       <c r="C388" t="inlineStr">
         <is>
-          <t>Oct-26</t>
+          <t>Nov-26</t>
         </is>
       </c>
       <c r="D388" s="2" t="n">
-        <v>46296</v>
+        <v>46327</v>
       </c>
       <c r="E388" t="inlineStr">
         <is>
@@ -19685,7 +19685,7 @@
       </c>
       <c r="F388" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>High</t>
         </is>
       </c>
     </row>
@@ -19702,11 +19702,11 @@
       </c>
       <c r="C389" t="inlineStr">
         <is>
-          <t>Nov-26</t>
+          <t>Dec-26</t>
         </is>
       </c>
       <c r="D389" s="2" t="n">
-        <v>46327</v>
+        <v>46357</v>
       </c>
       <c r="E389" t="inlineStr">
         <is>
@@ -19715,7 +19715,7 @@
       </c>
       <c r="F389" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>High</t>
         </is>
       </c>
     </row>
@@ -19732,11 +19732,11 @@
       </c>
       <c r="C390" t="inlineStr">
         <is>
-          <t>Dec-26</t>
+          <t>Jan-27</t>
         </is>
       </c>
       <c r="D390" s="2" t="n">
-        <v>46357</v>
+        <v>46388</v>
       </c>
       <c r="E390" t="inlineStr">
         <is>
@@ -19745,7 +19745,7 @@
       </c>
       <c r="F390" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>High</t>
         </is>
       </c>
     </row>
@@ -19762,11 +19762,11 @@
       </c>
       <c r="C391" t="inlineStr">
         <is>
-          <t>Jan-27</t>
+          <t>Feb-27</t>
         </is>
       </c>
       <c r="D391" s="2" t="n">
-        <v>46388</v>
+        <v>46419</v>
       </c>
       <c r="E391" t="inlineStr">
         <is>
@@ -19775,7 +19775,7 @@
       </c>
       <c r="F391" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>High</t>
         </is>
       </c>
     </row>
@@ -19792,11 +19792,11 @@
       </c>
       <c r="C392" t="inlineStr">
         <is>
-          <t>Feb-27</t>
+          <t>Mar-27</t>
         </is>
       </c>
       <c r="D392" s="2" t="n">
-        <v>46419</v>
+        <v>46447</v>
       </c>
       <c r="E392" t="inlineStr">
         <is>
@@ -19805,7 +19805,7 @@
       </c>
       <c r="F392" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>High</t>
         </is>
       </c>
     </row>
@@ -19822,11 +19822,11 @@
       </c>
       <c r="C393" t="inlineStr">
         <is>
-          <t>Sep-26</t>
+          <t>Oct-26</t>
         </is>
       </c>
       <c r="D393" s="2" t="n">
-        <v>46266</v>
+        <v>46296</v>
       </c>
       <c r="E393" t="inlineStr">
         <is>
@@ -19835,7 +19835,7 @@
       </c>
       <c r="F393" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>High</t>
         </is>
       </c>
     </row>
@@ -19852,11 +19852,11 @@
       </c>
       <c r="C394" t="inlineStr">
         <is>
-          <t>Oct-26</t>
+          <t>Nov-26</t>
         </is>
       </c>
       <c r="D394" s="2" t="n">
-        <v>46296</v>
+        <v>46327</v>
       </c>
       <c r="E394" t="inlineStr">
         <is>
@@ -19865,7 +19865,7 @@
       </c>
       <c r="F394" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>High</t>
         </is>
       </c>
     </row>
@@ -19882,11 +19882,11 @@
       </c>
       <c r="C395" t="inlineStr">
         <is>
-          <t>Nov-26</t>
+          <t>Dec-26</t>
         </is>
       </c>
       <c r="D395" s="2" t="n">
-        <v>46327</v>
+        <v>46357</v>
       </c>
       <c r="E395" t="inlineStr">
         <is>
@@ -19895,7 +19895,7 @@
       </c>
       <c r="F395" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>High</t>
         </is>
       </c>
     </row>
@@ -19912,11 +19912,11 @@
       </c>
       <c r="C396" t="inlineStr">
         <is>
-          <t>Dec-26</t>
+          <t>Jan-27</t>
         </is>
       </c>
       <c r="D396" s="2" t="n">
-        <v>46357</v>
+        <v>46388</v>
       </c>
       <c r="E396" t="inlineStr">
         <is>
@@ -19925,7 +19925,7 @@
       </c>
       <c r="F396" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>High</t>
         </is>
       </c>
     </row>
@@ -19942,11 +19942,11 @@
       </c>
       <c r="C397" t="inlineStr">
         <is>
-          <t>Jan-27</t>
+          <t>Feb-27</t>
         </is>
       </c>
       <c r="D397" s="2" t="n">
-        <v>46388</v>
+        <v>46419</v>
       </c>
       <c r="E397" t="inlineStr">
         <is>
@@ -19955,7 +19955,7 @@
       </c>
       <c r="F397" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>High</t>
         </is>
       </c>
     </row>
@@ -19972,11 +19972,11 @@
       </c>
       <c r="C398" t="inlineStr">
         <is>
-          <t>Feb-27</t>
+          <t>Mar-27</t>
         </is>
       </c>
       <c r="D398" s="2" t="n">
-        <v>46419</v>
+        <v>46447</v>
       </c>
       <c r="E398" t="inlineStr">
         <is>
@@ -19985,7 +19985,7 @@
       </c>
       <c r="F398" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>High</t>
         </is>
       </c>
     </row>
@@ -20002,11 +20002,11 @@
       </c>
       <c r="C399" t="inlineStr">
         <is>
-          <t>Sep-26</t>
+          <t>Oct-26</t>
         </is>
       </c>
       <c r="D399" s="2" t="n">
-        <v>46266</v>
+        <v>46296</v>
       </c>
       <c r="E399" t="inlineStr">
         <is>
@@ -20015,7 +20015,7 @@
       </c>
       <c r="F399" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>High</t>
         </is>
       </c>
     </row>
@@ -20032,11 +20032,11 @@
       </c>
       <c r="C400" t="inlineStr">
         <is>
-          <t>Oct-26</t>
+          <t>Nov-26</t>
         </is>
       </c>
       <c r="D400" s="2" t="n">
-        <v>46296</v>
+        <v>46327</v>
       </c>
       <c r="E400" t="inlineStr">
         <is>
@@ -20045,7 +20045,7 @@
       </c>
       <c r="F400" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>High</t>
         </is>
       </c>
     </row>
@@ -20062,11 +20062,11 @@
       </c>
       <c r="C401" t="inlineStr">
         <is>
-          <t>Nov-26</t>
+          <t>Dec-26</t>
         </is>
       </c>
       <c r="D401" s="2" t="n">
-        <v>46327</v>
+        <v>46357</v>
       </c>
       <c r="E401" t="inlineStr">
         <is>
@@ -20075,7 +20075,7 @@
       </c>
       <c r="F401" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>High</t>
         </is>
       </c>
     </row>
@@ -20092,11 +20092,11 @@
       </c>
       <c r="C402" t="inlineStr">
         <is>
-          <t>Dec-26</t>
+          <t>Jan-27</t>
         </is>
       </c>
       <c r="D402" s="2" t="n">
-        <v>46357</v>
+        <v>46388</v>
       </c>
       <c r="E402" t="inlineStr">
         <is>
@@ -20105,7 +20105,7 @@
       </c>
       <c r="F402" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>High</t>
         </is>
       </c>
     </row>
@@ -20122,11 +20122,11 @@
       </c>
       <c r="C403" t="inlineStr">
         <is>
-          <t>Jan-27</t>
+          <t>Feb-27</t>
         </is>
       </c>
       <c r="D403" s="2" t="n">
-        <v>46388</v>
+        <v>46419</v>
       </c>
       <c r="E403" t="inlineStr">
         <is>
@@ -20135,7 +20135,7 @@
       </c>
       <c r="F403" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>High</t>
         </is>
       </c>
     </row>
@@ -20152,11 +20152,11 @@
       </c>
       <c r="C404" t="inlineStr">
         <is>
-          <t>Feb-27</t>
+          <t>Mar-27</t>
         </is>
       </c>
       <c r="D404" s="2" t="n">
-        <v>46419</v>
+        <v>46447</v>
       </c>
       <c r="E404" t="inlineStr">
         <is>
@@ -20165,7 +20165,7 @@
       </c>
       <c r="F404" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>High</t>
         </is>
       </c>
     </row>
@@ -20182,11 +20182,11 @@
       </c>
       <c r="C405" t="inlineStr">
         <is>
-          <t>Sep-26</t>
+          <t>Oct-26</t>
         </is>
       </c>
       <c r="D405" s="2" t="n">
-        <v>46266</v>
+        <v>46296</v>
       </c>
       <c r="E405" t="inlineStr">
         <is>
@@ -20195,7 +20195,7 @@
       </c>
       <c r="F405" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>High</t>
         </is>
       </c>
     </row>
@@ -20212,11 +20212,11 @@
       </c>
       <c r="C406" t="inlineStr">
         <is>
-          <t>Oct-26</t>
+          <t>Nov-26</t>
         </is>
       </c>
       <c r="D406" s="2" t="n">
-        <v>46296</v>
+        <v>46327</v>
       </c>
       <c r="E406" t="inlineStr">
         <is>
@@ -20225,7 +20225,7 @@
       </c>
       <c r="F406" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>High</t>
         </is>
       </c>
     </row>
@@ -20242,11 +20242,11 @@
       </c>
       <c r="C407" t="inlineStr">
         <is>
-          <t>Nov-26</t>
+          <t>Dec-26</t>
         </is>
       </c>
       <c r="D407" s="2" t="n">
-        <v>46327</v>
+        <v>46357</v>
       </c>
       <c r="E407" t="inlineStr">
         <is>
@@ -20255,7 +20255,7 @@
       </c>
       <c r="F407" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>High</t>
         </is>
       </c>
     </row>
@@ -20272,11 +20272,11 @@
       </c>
       <c r="C408" t="inlineStr">
         <is>
-          <t>Dec-26</t>
+          <t>Jan-27</t>
         </is>
       </c>
       <c r="D408" s="2" t="n">
-        <v>46357</v>
+        <v>46388</v>
       </c>
       <c r="E408" t="inlineStr">
         <is>
@@ -20285,7 +20285,7 @@
       </c>
       <c r="F408" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>High</t>
         </is>
       </c>
     </row>
@@ -20302,11 +20302,11 @@
       </c>
       <c r="C409" t="inlineStr">
         <is>
-          <t>Jan-27</t>
+          <t>Feb-27</t>
         </is>
       </c>
       <c r="D409" s="2" t="n">
-        <v>46388</v>
+        <v>46419</v>
       </c>
       <c r="E409" t="inlineStr">
         <is>
@@ -20315,7 +20315,7 @@
       </c>
       <c r="F409" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>High</t>
         </is>
       </c>
     </row>
@@ -20332,11 +20332,11 @@
       </c>
       <c r="C410" t="inlineStr">
         <is>
-          <t>Feb-27</t>
+          <t>Mar-27</t>
         </is>
       </c>
       <c r="D410" s="2" t="n">
-        <v>46419</v>
+        <v>46447</v>
       </c>
       <c r="E410" t="inlineStr">
         <is>
@@ -20345,7 +20345,7 @@
       </c>
       <c r="F410" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>High</t>
         </is>
       </c>
     </row>
@@ -20362,11 +20362,11 @@
       </c>
       <c r="C411" t="inlineStr">
         <is>
-          <t>Oct-26</t>
+          <t>Nov-26</t>
         </is>
       </c>
       <c r="D411" s="2" t="n">
-        <v>46296</v>
+        <v>46327</v>
       </c>
       <c r="E411" t="inlineStr">
         <is>
@@ -20375,7 +20375,7 @@
       </c>
       <c r="F411" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>High</t>
         </is>
       </c>
     </row>
@@ -20392,11 +20392,11 @@
       </c>
       <c r="C412" t="inlineStr">
         <is>
-          <t>Nov-26</t>
+          <t>Dec-26</t>
         </is>
       </c>
       <c r="D412" s="2" t="n">
-        <v>46327</v>
+        <v>46357</v>
       </c>
       <c r="E412" t="inlineStr">
         <is>
@@ -20405,7 +20405,7 @@
       </c>
       <c r="F412" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>High</t>
         </is>
       </c>
     </row>
@@ -20422,11 +20422,11 @@
       </c>
       <c r="C413" t="inlineStr">
         <is>
-          <t>Dec-26</t>
+          <t>Jan-27</t>
         </is>
       </c>
       <c r="D413" s="2" t="n">
-        <v>46357</v>
+        <v>46388</v>
       </c>
       <c r="E413" t="inlineStr">
         <is>
@@ -20435,7 +20435,7 @@
       </c>
       <c r="F413" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>High</t>
         </is>
       </c>
     </row>
@@ -20452,11 +20452,11 @@
       </c>
       <c r="C414" t="inlineStr">
         <is>
-          <t>Jan-27</t>
+          <t>Feb-27</t>
         </is>
       </c>
       <c r="D414" s="2" t="n">
-        <v>46388</v>
+        <v>46419</v>
       </c>
       <c r="E414" t="inlineStr">
         <is>
@@ -20465,7 +20465,7 @@
       </c>
       <c r="F414" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>High</t>
         </is>
       </c>
     </row>
@@ -20482,11 +20482,11 @@
       </c>
       <c r="C415" t="inlineStr">
         <is>
-          <t>Feb-27</t>
+          <t>Mar-27</t>
         </is>
       </c>
       <c r="D415" s="2" t="n">
-        <v>46419</v>
+        <v>46447</v>
       </c>
       <c r="E415" t="inlineStr">
         <is>
@@ -20495,7 +20495,7 @@
       </c>
       <c r="F415" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>High</t>
         </is>
       </c>
     </row>
@@ -20512,11 +20512,11 @@
       </c>
       <c r="C416" t="inlineStr">
         <is>
-          <t>Mar-27</t>
+          <t>Apr-27</t>
         </is>
       </c>
       <c r="D416" s="2" t="n">
-        <v>46447</v>
+        <v>46478</v>
       </c>
       <c r="E416" t="inlineStr">
         <is>
@@ -20525,7 +20525,7 @@
       </c>
       <c r="F416" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>High</t>
         </is>
       </c>
     </row>
@@ -20542,11 +20542,11 @@
       </c>
       <c r="C417" t="inlineStr">
         <is>
-          <t>Oct-26</t>
+          <t>Nov-26</t>
         </is>
       </c>
       <c r="D417" s="2" t="n">
-        <v>46296</v>
+        <v>46327</v>
       </c>
       <c r="E417" t="inlineStr">
         <is>
@@ -20555,7 +20555,7 @@
       </c>
       <c r="F417" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>High</t>
         </is>
       </c>
     </row>
@@ -20572,11 +20572,11 @@
       </c>
       <c r="C418" t="inlineStr">
         <is>
-          <t>Nov-26</t>
+          <t>Dec-26</t>
         </is>
       </c>
       <c r="D418" s="2" t="n">
-        <v>46327</v>
+        <v>46357</v>
       </c>
       <c r="E418" t="inlineStr">
         <is>
@@ -20585,7 +20585,7 @@
       </c>
       <c r="F418" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>High</t>
         </is>
       </c>
     </row>
@@ -20602,11 +20602,11 @@
       </c>
       <c r="C419" t="inlineStr">
         <is>
-          <t>Dec-26</t>
+          <t>Jan-27</t>
         </is>
       </c>
       <c r="D419" s="2" t="n">
-        <v>46357</v>
+        <v>46388</v>
       </c>
       <c r="E419" t="inlineStr">
         <is>
@@ -20615,7 +20615,7 @@
       </c>
       <c r="F419" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>High</t>
         </is>
       </c>
     </row>
@@ -20632,11 +20632,11 @@
       </c>
       <c r="C420" t="inlineStr">
         <is>
-          <t>Jan-27</t>
+          <t>Feb-27</t>
         </is>
       </c>
       <c r="D420" s="2" t="n">
-        <v>46388</v>
+        <v>46419</v>
       </c>
       <c r="E420" t="inlineStr">
         <is>
@@ -20645,7 +20645,7 @@
       </c>
       <c r="F420" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>High</t>
         </is>
       </c>
     </row>
@@ -20662,11 +20662,11 @@
       </c>
       <c r="C421" t="inlineStr">
         <is>
-          <t>Feb-27</t>
+          <t>Mar-27</t>
         </is>
       </c>
       <c r="D421" s="2" t="n">
-        <v>46419</v>
+        <v>46447</v>
       </c>
       <c r="E421" t="inlineStr">
         <is>
@@ -20675,7 +20675,7 @@
       </c>
       <c r="F421" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>High</t>
         </is>
       </c>
     </row>
@@ -20692,11 +20692,11 @@
       </c>
       <c r="C422" t="inlineStr">
         <is>
-          <t>Mar-27</t>
+          <t>Apr-27</t>
         </is>
       </c>
       <c r="D422" s="2" t="n">
-        <v>46447</v>
+        <v>46478</v>
       </c>
       <c r="E422" t="inlineStr">
         <is>
@@ -20705,7 +20705,7 @@
       </c>
       <c r="F422" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>High</t>
         </is>
       </c>
     </row>
@@ -20722,11 +20722,11 @@
       </c>
       <c r="C423" t="inlineStr">
         <is>
-          <t>Oct-26</t>
+          <t>Nov-26</t>
         </is>
       </c>
       <c r="D423" s="2" t="n">
-        <v>46296</v>
+        <v>46327</v>
       </c>
       <c r="E423" t="inlineStr">
         <is>
@@ -20735,7 +20735,7 @@
       </c>
       <c r="F423" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>High</t>
         </is>
       </c>
     </row>
@@ -20752,11 +20752,11 @@
       </c>
       <c r="C424" t="inlineStr">
         <is>
-          <t>Nov-26</t>
+          <t>Dec-26</t>
         </is>
       </c>
       <c r="D424" s="2" t="n">
-        <v>46327</v>
+        <v>46357</v>
       </c>
       <c r="E424" t="inlineStr">
         <is>
@@ -20765,7 +20765,7 @@
       </c>
       <c r="F424" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>High</t>
         </is>
       </c>
     </row>
@@ -20782,11 +20782,11 @@
       </c>
       <c r="C425" t="inlineStr">
         <is>
-          <t>Dec-26</t>
+          <t>Jan-27</t>
         </is>
       </c>
       <c r="D425" s="2" t="n">
-        <v>46357</v>
+        <v>46388</v>
       </c>
       <c r="E425" t="inlineStr">
         <is>
@@ -20795,7 +20795,7 @@
       </c>
       <c r="F425" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>High</t>
         </is>
       </c>
     </row>
@@ -20812,11 +20812,11 @@
       </c>
       <c r="C426" t="inlineStr">
         <is>
-          <t>Jan-27</t>
+          <t>Feb-27</t>
         </is>
       </c>
       <c r="D426" s="2" t="n">
-        <v>46388</v>
+        <v>46419</v>
       </c>
       <c r="E426" t="inlineStr">
         <is>
@@ -20825,7 +20825,7 @@
       </c>
       <c r="F426" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>High</t>
         </is>
       </c>
     </row>
@@ -20842,11 +20842,11 @@
       </c>
       <c r="C427" t="inlineStr">
         <is>
-          <t>Feb-27</t>
+          <t>Mar-27</t>
         </is>
       </c>
       <c r="D427" s="2" t="n">
-        <v>46419</v>
+        <v>46447</v>
       </c>
       <c r="E427" t="inlineStr">
         <is>
@@ -20855,7 +20855,7 @@
       </c>
       <c r="F427" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>High</t>
         </is>
       </c>
     </row>
@@ -20872,11 +20872,11 @@
       </c>
       <c r="C428" t="inlineStr">
         <is>
-          <t>Mar-27</t>
+          <t>Apr-27</t>
         </is>
       </c>
       <c r="D428" s="2" t="n">
-        <v>46447</v>
+        <v>46478</v>
       </c>
       <c r="E428" t="inlineStr">
         <is>
@@ -20885,7 +20885,7 @@
       </c>
       <c r="F428" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>High</t>
         </is>
       </c>
     </row>
@@ -20902,11 +20902,11 @@
       </c>
       <c r="C429" t="inlineStr">
         <is>
-          <t>Apr-27</t>
+          <t>May-27</t>
         </is>
       </c>
       <c r="D429" s="2" t="n">
-        <v>46478</v>
+        <v>46508</v>
       </c>
       <c r="E429" t="inlineStr">
         <is>
@@ -20915,7 +20915,7 @@
       </c>
       <c r="F429" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>High</t>
         </is>
       </c>
     </row>
@@ -20932,11 +20932,11 @@
       </c>
       <c r="C430" t="inlineStr">
         <is>
-          <t>May-27</t>
+          <t>Jun-27</t>
         </is>
       </c>
       <c r="D430" s="2" t="n">
-        <v>46508</v>
+        <v>46539</v>
       </c>
       <c r="E430" t="inlineStr">
         <is>
@@ -20945,7 +20945,7 @@
       </c>
       <c r="F430" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>High</t>
         </is>
       </c>
     </row>
@@ -20962,11 +20962,11 @@
       </c>
       <c r="C431" t="inlineStr">
         <is>
-          <t>Nov-26</t>
+          <t>Dec-26</t>
         </is>
       </c>
       <c r="D431" s="2" t="n">
-        <v>46327</v>
+        <v>46357</v>
       </c>
       <c r="E431" t="inlineStr">
         <is>
@@ -20975,7 +20975,7 @@
       </c>
       <c r="F431" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>High</t>
         </is>
       </c>
     </row>
@@ -20992,11 +20992,11 @@
       </c>
       <c r="C432" t="inlineStr">
         <is>
-          <t>Dec-26</t>
+          <t>Jan-27</t>
         </is>
       </c>
       <c r="D432" s="2" t="n">
-        <v>46357</v>
+        <v>46388</v>
       </c>
       <c r="E432" t="inlineStr">
         <is>
@@ -21005,7 +21005,7 @@
       </c>
       <c r="F432" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>High</t>
         </is>
       </c>
     </row>
@@ -21022,11 +21022,11 @@
       </c>
       <c r="C433" t="inlineStr">
         <is>
-          <t>Jan-27</t>
+          <t>Feb-27</t>
         </is>
       </c>
       <c r="D433" s="2" t="n">
-        <v>46388</v>
+        <v>46419</v>
       </c>
       <c r="E433" t="inlineStr">
         <is>
@@ -21035,7 +21035,7 @@
       </c>
       <c r="F433" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>High</t>
         </is>
       </c>
     </row>
@@ -21052,11 +21052,11 @@
       </c>
       <c r="C434" t="inlineStr">
         <is>
-          <t>Feb-27</t>
+          <t>Mar-27</t>
         </is>
       </c>
       <c r="D434" s="2" t="n">
-        <v>46419</v>
+        <v>46447</v>
       </c>
       <c r="E434" t="inlineStr">
         <is>
@@ -21065,7 +21065,7 @@
       </c>
       <c r="F434" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>High</t>
         </is>
       </c>
     </row>
@@ -21082,11 +21082,11 @@
       </c>
       <c r="C435" t="inlineStr">
         <is>
-          <t>Mar-27</t>
+          <t>Apr-27</t>
         </is>
       </c>
       <c r="D435" s="2" t="n">
-        <v>46447</v>
+        <v>46478</v>
       </c>
       <c r="E435" t="inlineStr">
         <is>
@@ -21095,7 +21095,7 @@
       </c>
       <c r="F435" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>High</t>
         </is>
       </c>
     </row>
@@ -21112,11 +21112,11 @@
       </c>
       <c r="C436" t="inlineStr">
         <is>
-          <t>Apr-27</t>
+          <t>May-27</t>
         </is>
       </c>
       <c r="D436" s="2" t="n">
-        <v>46478</v>
+        <v>46508</v>
       </c>
       <c r="E436" t="inlineStr">
         <is>
@@ -21125,7 +21125,7 @@
       </c>
       <c r="F436" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>High</t>
         </is>
       </c>
     </row>
@@ -21142,11 +21142,11 @@
       </c>
       <c r="C437" t="inlineStr">
         <is>
-          <t>May-27</t>
+          <t>Jun-27</t>
         </is>
       </c>
       <c r="D437" s="2" t="n">
-        <v>46508</v>
+        <v>46539</v>
       </c>
       <c r="E437" t="inlineStr">
         <is>
@@ -21155,7 +21155,7 @@
       </c>
       <c r="F437" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>High</t>
         </is>
       </c>
     </row>
@@ -21172,11 +21172,11 @@
       </c>
       <c r="C438" t="inlineStr">
         <is>
-          <t>Nov-26</t>
+          <t>Dec-26</t>
         </is>
       </c>
       <c r="D438" s="2" t="n">
-        <v>46327</v>
+        <v>46357</v>
       </c>
       <c r="E438" t="inlineStr">
         <is>
@@ -21185,7 +21185,7 @@
       </c>
       <c r="F438" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>High</t>
         </is>
       </c>
     </row>
@@ -21202,11 +21202,11 @@
       </c>
       <c r="C439" t="inlineStr">
         <is>
-          <t>Dec-26</t>
+          <t>Jan-27</t>
         </is>
       </c>
       <c r="D439" s="2" t="n">
-        <v>46357</v>
+        <v>46388</v>
       </c>
       <c r="E439" t="inlineStr">
         <is>
@@ -21215,7 +21215,7 @@
       </c>
       <c r="F439" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>High</t>
         </is>
       </c>
     </row>
@@ -21232,11 +21232,11 @@
       </c>
       <c r="C440" t="inlineStr">
         <is>
-          <t>Jan-27</t>
+          <t>Feb-27</t>
         </is>
       </c>
       <c r="D440" s="2" t="n">
-        <v>46388</v>
+        <v>46419</v>
       </c>
       <c r="E440" t="inlineStr">
         <is>
@@ -21245,7 +21245,7 @@
       </c>
       <c r="F440" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>High</t>
         </is>
       </c>
     </row>
@@ -21262,11 +21262,11 @@
       </c>
       <c r="C441" t="inlineStr">
         <is>
-          <t>Feb-27</t>
+          <t>Mar-27</t>
         </is>
       </c>
       <c r="D441" s="2" t="n">
-        <v>46419</v>
+        <v>46447</v>
       </c>
       <c r="E441" t="inlineStr">
         <is>
@@ -21275,7 +21275,7 @@
       </c>
       <c r="F441" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>High</t>
         </is>
       </c>
     </row>
@@ -21292,11 +21292,11 @@
       </c>
       <c r="C442" t="inlineStr">
         <is>
-          <t>Mar-27</t>
+          <t>Apr-27</t>
         </is>
       </c>
       <c r="D442" s="2" t="n">
-        <v>46447</v>
+        <v>46478</v>
       </c>
       <c r="E442" t="inlineStr">
         <is>
@@ -21305,7 +21305,7 @@
       </c>
       <c r="F442" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>High</t>
         </is>
       </c>
     </row>
@@ -21322,11 +21322,11 @@
       </c>
       <c r="C443" t="inlineStr">
         <is>
-          <t>Apr-27</t>
+          <t>May-27</t>
         </is>
       </c>
       <c r="D443" s="2" t="n">
-        <v>46478</v>
+        <v>46508</v>
       </c>
       <c r="E443" t="inlineStr">
         <is>
@@ -21335,7 +21335,7 @@
       </c>
       <c r="F443" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>High</t>
         </is>
       </c>
     </row>
@@ -21352,11 +21352,11 @@
       </c>
       <c r="C444" t="inlineStr">
         <is>
-          <t>May-27</t>
+          <t>Jun-27</t>
         </is>
       </c>
       <c r="D444" s="2" t="n">
-        <v>46508</v>
+        <v>46539</v>
       </c>
       <c r="E444" t="inlineStr">
         <is>
@@ -21365,7 +21365,7 @@
       </c>
       <c r="F444" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>High</t>
         </is>
       </c>
     </row>
@@ -21382,11 +21382,11 @@
       </c>
       <c r="C445" t="inlineStr">
         <is>
-          <t>Jun-27</t>
+          <t>Jul-27</t>
         </is>
       </c>
       <c r="D445" s="2" t="n">
-        <v>46539</v>
+        <v>46569</v>
       </c>
       <c r="E445" t="inlineStr">
         <is>
@@ -21395,7 +21395,7 @@
       </c>
       <c r="F445" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>High</t>
         </is>
       </c>
     </row>
@@ -21412,11 +21412,11 @@
       </c>
       <c r="C446" t="inlineStr">
         <is>
-          <t>Jul-27</t>
+          <t>Aug-27</t>
         </is>
       </c>
       <c r="D446" s="2" t="n">
-        <v>46569</v>
+        <v>46600</v>
       </c>
       <c r="E446" t="inlineStr">
         <is>
@@ -21425,7 +21425,7 @@
       </c>
       <c r="F446" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>High</t>
         </is>
       </c>
     </row>
@@ -21442,11 +21442,11 @@
       </c>
       <c r="C447" t="inlineStr">
         <is>
-          <t>Aug-27</t>
+          <t>Sep-27</t>
         </is>
       </c>
       <c r="D447" s="2" t="n">
-        <v>46600</v>
+        <v>46631</v>
       </c>
       <c r="E447" t="inlineStr">
         <is>
@@ -21455,7 +21455,7 @@
       </c>
       <c r="F447" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>High</t>
         </is>
       </c>
     </row>
@@ -21472,11 +21472,11 @@
       </c>
       <c r="C448" t="inlineStr">
         <is>
-          <t>Sep-26</t>
+          <t>Oct-26</t>
         </is>
       </c>
       <c r="D448" s="2" t="n">
-        <v>46266</v>
+        <v>46296</v>
       </c>
       <c r="E448" t="inlineStr">
         <is>
@@ -21485,7 +21485,7 @@
       </c>
       <c r="F448" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>High</t>
         </is>
       </c>
     </row>
@@ -21502,11 +21502,11 @@
       </c>
       <c r="C449" t="inlineStr">
         <is>
-          <t>Oct-26</t>
+          <t>Nov-26</t>
         </is>
       </c>
       <c r="D449" s="2" t="n">
-        <v>46296</v>
+        <v>46327</v>
       </c>
       <c r="E449" t="inlineStr">
         <is>
@@ -21515,7 +21515,7 @@
       </c>
       <c r="F449" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>High</t>
         </is>
       </c>
     </row>
@@ -21532,11 +21532,11 @@
       </c>
       <c r="C450" t="inlineStr">
         <is>
-          <t>Nov-26</t>
+          <t>Dec-26</t>
         </is>
       </c>
       <c r="D450" s="2" t="n">
-        <v>46327</v>
+        <v>46357</v>
       </c>
       <c r="E450" t="inlineStr">
         <is>
@@ -21545,7 +21545,7 @@
       </c>
       <c r="F450" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>High</t>
         </is>
       </c>
     </row>
@@ -21562,11 +21562,11 @@
       </c>
       <c r="C451" t="inlineStr">
         <is>
-          <t>Dec-26</t>
+          <t>Jan-27</t>
         </is>
       </c>
       <c r="D451" s="2" t="n">
-        <v>46357</v>
+        <v>46388</v>
       </c>
       <c r="E451" t="inlineStr">
         <is>
@@ -21575,7 +21575,7 @@
       </c>
       <c r="F451" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>High</t>
         </is>
       </c>
     </row>
@@ -21592,11 +21592,11 @@
       </c>
       <c r="C452" t="inlineStr">
         <is>
-          <t>Jan-27</t>
+          <t>Feb-27</t>
         </is>
       </c>
       <c r="D452" s="2" t="n">
-        <v>46388</v>
+        <v>46419</v>
       </c>
       <c r="E452" t="inlineStr">
         <is>
@@ -21605,7 +21605,7 @@
       </c>
       <c r="F452" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>High</t>
         </is>
       </c>
     </row>
@@ -21622,11 +21622,11 @@
       </c>
       <c r="C453" t="inlineStr">
         <is>
-          <t>Feb-27</t>
+          <t>Mar-27</t>
         </is>
       </c>
       <c r="D453" s="2" t="n">
-        <v>46419</v>
+        <v>46447</v>
       </c>
       <c r="E453" t="inlineStr">
         <is>
@@ -21635,7 +21635,7 @@
       </c>
       <c r="F453" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>High</t>
         </is>
       </c>
     </row>
@@ -21652,11 +21652,11 @@
       </c>
       <c r="C454" t="inlineStr">
         <is>
-          <t>Dec-26</t>
+          <t>Jan-27</t>
         </is>
       </c>
       <c r="D454" s="2" t="n">
-        <v>46357</v>
+        <v>46388</v>
       </c>
       <c r="E454" t="inlineStr">
         <is>
@@ -21665,7 +21665,7 @@
       </c>
       <c r="F454" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>High</t>
         </is>
       </c>
     </row>
@@ -21682,11 +21682,11 @@
       </c>
       <c r="C455" t="inlineStr">
         <is>
-          <t>Jan-27</t>
+          <t>Feb-27</t>
         </is>
       </c>
       <c r="D455" s="2" t="n">
-        <v>46388</v>
+        <v>46419</v>
       </c>
       <c r="E455" t="inlineStr">
         <is>
@@ -21695,7 +21695,7 @@
       </c>
       <c r="F455" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>High</t>
         </is>
       </c>
     </row>
@@ -21712,11 +21712,11 @@
       </c>
       <c r="C456" t="inlineStr">
         <is>
-          <t>Feb-27</t>
+          <t>Mar-27</t>
         </is>
       </c>
       <c r="D456" s="2" t="n">
-        <v>46419</v>
+        <v>46447</v>
       </c>
       <c r="E456" t="inlineStr">
         <is>
@@ -21725,7 +21725,7 @@
       </c>
       <c r="F456" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>High</t>
         </is>
       </c>
     </row>
@@ -21742,11 +21742,11 @@
       </c>
       <c r="C457" t="inlineStr">
         <is>
-          <t>Mar-27</t>
+          <t>Apr-27</t>
         </is>
       </c>
       <c r="D457" s="2" t="n">
-        <v>46447</v>
+        <v>46478</v>
       </c>
       <c r="E457" t="inlineStr">
         <is>
@@ -21755,7 +21755,7 @@
       </c>
       <c r="F457" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>High</t>
         </is>
       </c>
     </row>
@@ -21772,11 +21772,11 @@
       </c>
       <c r="C458" t="inlineStr">
         <is>
-          <t>Apr-27</t>
+          <t>May-27</t>
         </is>
       </c>
       <c r="D458" s="2" t="n">
-        <v>46478</v>
+        <v>46508</v>
       </c>
       <c r="E458" t="inlineStr">
         <is>
@@ -21785,7 +21785,7 @@
       </c>
       <c r="F458" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>High</t>
         </is>
       </c>
     </row>
@@ -21802,11 +21802,11 @@
       </c>
       <c r="C459" t="inlineStr">
         <is>
-          <t>May-27</t>
+          <t>Jun-27</t>
         </is>
       </c>
       <c r="D459" s="2" t="n">
-        <v>46508</v>
+        <v>46539</v>
       </c>
       <c r="E459" t="inlineStr">
         <is>
@@ -21815,7 +21815,7 @@
       </c>
       <c r="F459" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>High</t>
         </is>
       </c>
     </row>
@@ -21832,11 +21832,11 @@
       </c>
       <c r="C460" t="inlineStr">
         <is>
-          <t>Jun-27</t>
+          <t>Jul-27</t>
         </is>
       </c>
       <c r="D460" s="2" t="n">
-        <v>46539</v>
+        <v>46569</v>
       </c>
       <c r="E460" t="inlineStr">
         <is>
@@ -21845,7 +21845,7 @@
       </c>
       <c r="F460" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>High</t>
         </is>
       </c>
     </row>
@@ -21862,11 +21862,11 @@
       </c>
       <c r="C461" t="inlineStr">
         <is>
-          <t>Dec-26</t>
+          <t>Jan-27</t>
         </is>
       </c>
       <c r="D461" s="2" t="n">
-        <v>46357</v>
+        <v>46388</v>
       </c>
       <c r="E461" t="inlineStr">
         <is>
@@ -21875,7 +21875,7 @@
       </c>
       <c r="F461" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>High</t>
         </is>
       </c>
     </row>
@@ -21892,11 +21892,11 @@
       </c>
       <c r="C462" t="inlineStr">
         <is>
-          <t>Jan-27</t>
+          <t>Feb-27</t>
         </is>
       </c>
       <c r="D462" s="2" t="n">
-        <v>46388</v>
+        <v>46419</v>
       </c>
       <c r="E462" t="inlineStr">
         <is>
@@ -21905,7 +21905,7 @@
       </c>
       <c r="F462" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>High</t>
         </is>
       </c>
     </row>
@@ -21922,11 +21922,11 @@
       </c>
       <c r="C463" t="inlineStr">
         <is>
-          <t>Feb-27</t>
+          <t>Mar-27</t>
         </is>
       </c>
       <c r="D463" s="2" t="n">
-        <v>46419</v>
+        <v>46447</v>
       </c>
       <c r="E463" t="inlineStr">
         <is>
@@ -21935,7 +21935,7 @@
       </c>
       <c r="F463" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>High</t>
         </is>
       </c>
     </row>
@@ -21952,11 +21952,11 @@
       </c>
       <c r="C464" t="inlineStr">
         <is>
-          <t>Mar-27</t>
+          <t>Apr-27</t>
         </is>
       </c>
       <c r="D464" s="2" t="n">
-        <v>46447</v>
+        <v>46478</v>
       </c>
       <c r="E464" t="inlineStr">
         <is>
@@ -21965,7 +21965,7 @@
       </c>
       <c r="F464" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>High</t>
         </is>
       </c>
     </row>
@@ -21982,11 +21982,11 @@
       </c>
       <c r="C465" t="inlineStr">
         <is>
-          <t>Apr-27</t>
+          <t>May-27</t>
         </is>
       </c>
       <c r="D465" s="2" t="n">
-        <v>46478</v>
+        <v>46508</v>
       </c>
       <c r="E465" t="inlineStr">
         <is>
@@ -21995,7 +21995,7 @@
       </c>
       <c r="F465" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>High</t>
         </is>
       </c>
     </row>
@@ -22012,11 +22012,11 @@
       </c>
       <c r="C466" t="inlineStr">
         <is>
-          <t>May-27</t>
+          <t>Jun-27</t>
         </is>
       </c>
       <c r="D466" s="2" t="n">
-        <v>46508</v>
+        <v>46539</v>
       </c>
       <c r="E466" t="inlineStr">
         <is>
@@ -22025,7 +22025,7 @@
       </c>
       <c r="F466" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>High</t>
         </is>
       </c>
     </row>
@@ -22042,11 +22042,11 @@
       </c>
       <c r="C467" t="inlineStr">
         <is>
-          <t>Jun-27</t>
+          <t>Jul-27</t>
         </is>
       </c>
       <c r="D467" s="2" t="n">
-        <v>46539</v>
+        <v>46569</v>
       </c>
       <c r="E467" t="inlineStr">
         <is>
@@ -22055,7 +22055,7 @@
       </c>
       <c r="F467" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>High</t>
         </is>
       </c>
     </row>
@@ -22072,11 +22072,11 @@
       </c>
       <c r="C468" t="inlineStr">
         <is>
-          <t>Dec-26</t>
+          <t>Jan-27</t>
         </is>
       </c>
       <c r="D468" s="2" t="n">
-        <v>46357</v>
+        <v>46388</v>
       </c>
       <c r="E468" t="inlineStr">
         <is>
@@ -22085,7 +22085,7 @@
       </c>
       <c r="F468" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>High</t>
         </is>
       </c>
     </row>
@@ -22102,11 +22102,11 @@
       </c>
       <c r="C469" t="inlineStr">
         <is>
-          <t>Jan-27</t>
+          <t>Feb-27</t>
         </is>
       </c>
       <c r="D469" s="2" t="n">
-        <v>46388</v>
+        <v>46419</v>
       </c>
       <c r="E469" t="inlineStr">
         <is>
@@ -22115,7 +22115,7 @@
       </c>
       <c r="F469" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>High</t>
         </is>
       </c>
     </row>
@@ -22132,11 +22132,11 @@
       </c>
       <c r="C470" t="inlineStr">
         <is>
-          <t>Feb-27</t>
+          <t>Mar-27</t>
         </is>
       </c>
       <c r="D470" s="2" t="n">
-        <v>46419</v>
+        <v>46447</v>
       </c>
       <c r="E470" t="inlineStr">
         <is>
@@ -22145,7 +22145,7 @@
       </c>
       <c r="F470" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>High</t>
         </is>
       </c>
     </row>
@@ -22162,11 +22162,11 @@
       </c>
       <c r="C471" t="inlineStr">
         <is>
-          <t>Mar-27</t>
+          <t>Apr-27</t>
         </is>
       </c>
       <c r="D471" s="2" t="n">
-        <v>46447</v>
+        <v>46478</v>
       </c>
       <c r="E471" t="inlineStr">
         <is>
@@ -22175,7 +22175,7 @@
       </c>
       <c r="F471" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>High</t>
         </is>
       </c>
     </row>
@@ -22192,11 +22192,11 @@
       </c>
       <c r="C472" t="inlineStr">
         <is>
-          <t>Apr-27</t>
+          <t>May-27</t>
         </is>
       </c>
       <c r="D472" s="2" t="n">
-        <v>46478</v>
+        <v>46508</v>
       </c>
       <c r="E472" t="inlineStr">
         <is>
@@ -22205,7 +22205,7 @@
       </c>
       <c r="F472" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>High</t>
         </is>
       </c>
     </row>
@@ -22222,11 +22222,11 @@
       </c>
       <c r="C473" t="inlineStr">
         <is>
-          <t>May-27</t>
+          <t>Jun-27</t>
         </is>
       </c>
       <c r="D473" s="2" t="n">
-        <v>46508</v>
+        <v>46539</v>
       </c>
       <c r="E473" t="inlineStr">
         <is>
@@ -22235,7 +22235,7 @@
       </c>
       <c r="F473" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>High</t>
         </is>
       </c>
     </row>
@@ -22252,11 +22252,11 @@
       </c>
       <c r="C474" t="inlineStr">
         <is>
-          <t>Jun-27</t>
+          <t>Jul-27</t>
         </is>
       </c>
       <c r="D474" s="2" t="n">
-        <v>46539</v>
+        <v>46569</v>
       </c>
       <c r="E474" t="inlineStr">
         <is>
@@ -22265,7 +22265,7 @@
       </c>
       <c r="F474" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>High</t>
         </is>
       </c>
     </row>
@@ -22282,11 +22282,11 @@
       </c>
       <c r="C475" t="inlineStr">
         <is>
-          <t>Jan-27</t>
+          <t>Feb-27</t>
         </is>
       </c>
       <c r="D475" s="2" t="n">
-        <v>46388</v>
+        <v>46419</v>
       </c>
       <c r="E475" t="inlineStr">
         <is>
@@ -22295,7 +22295,7 @@
       </c>
       <c r="F475" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>High</t>
         </is>
       </c>
     </row>
@@ -22312,11 +22312,11 @@
       </c>
       <c r="C476" t="inlineStr">
         <is>
-          <t>Feb-27</t>
+          <t>Mar-27</t>
         </is>
       </c>
       <c r="D476" s="2" t="n">
-        <v>46419</v>
+        <v>46447</v>
       </c>
       <c r="E476" t="inlineStr">
         <is>
@@ -22325,7 +22325,7 @@
       </c>
       <c r="F476" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>High</t>
         </is>
       </c>
     </row>
@@ -22342,11 +22342,11 @@
       </c>
       <c r="C477" t="inlineStr">
         <is>
-          <t>Mar-27</t>
+          <t>Apr-27</t>
         </is>
       </c>
       <c r="D477" s="2" t="n">
-        <v>46447</v>
+        <v>46478</v>
       </c>
       <c r="E477" t="inlineStr">
         <is>
@@ -22355,7 +22355,7 @@
       </c>
       <c r="F477" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>High</t>
         </is>
       </c>
     </row>
@@ -22372,11 +22372,11 @@
       </c>
       <c r="C478" t="inlineStr">
         <is>
-          <t>Apr-27</t>
+          <t>May-27</t>
         </is>
       </c>
       <c r="D478" s="2" t="n">
-        <v>46478</v>
+        <v>46508</v>
       </c>
       <c r="E478" t="inlineStr">
         <is>
@@ -22385,7 +22385,7 @@
       </c>
       <c r="F478" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>High</t>
         </is>
       </c>
     </row>
@@ -22402,11 +22402,11 @@
       </c>
       <c r="C479" t="inlineStr">
         <is>
-          <t>May-27</t>
+          <t>Jun-27</t>
         </is>
       </c>
       <c r="D479" s="2" t="n">
-        <v>46508</v>
+        <v>46539</v>
       </c>
       <c r="E479" t="inlineStr">
         <is>
@@ -22415,7 +22415,7 @@
       </c>
       <c r="F479" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>High</t>
         </is>
       </c>
     </row>
@@ -22432,11 +22432,11 @@
       </c>
       <c r="C480" t="inlineStr">
         <is>
-          <t>Jun-27</t>
+          <t>Jul-27</t>
         </is>
       </c>
       <c r="D480" s="2" t="n">
-        <v>46539</v>
+        <v>46569</v>
       </c>
       <c r="E480" t="inlineStr">
         <is>
@@ -22445,7 +22445,7 @@
       </c>
       <c r="F480" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>High</t>
         </is>
       </c>
     </row>
@@ -22462,11 +22462,11 @@
       </c>
       <c r="C481" t="inlineStr">
         <is>
-          <t>Jul-27</t>
+          <t>Aug-27</t>
         </is>
       </c>
       <c r="D481" s="2" t="n">
-        <v>46569</v>
+        <v>46600</v>
       </c>
       <c r="E481" t="inlineStr">
         <is>
@@ -22475,7 +22475,7 @@
       </c>
       <c r="F481" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>High</t>
         </is>
       </c>
     </row>
@@ -22492,11 +22492,11 @@
       </c>
       <c r="C482" t="inlineStr">
         <is>
-          <t>Aug-27</t>
+          <t>Sep-27</t>
         </is>
       </c>
       <c r="D482" s="2" t="n">
-        <v>46600</v>
+        <v>46631</v>
       </c>
       <c r="E482" t="inlineStr">
         <is>
@@ -22505,7 +22505,7 @@
       </c>
       <c r="F482" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>High</t>
         </is>
       </c>
     </row>
@@ -22522,11 +22522,11 @@
       </c>
       <c r="C483" t="inlineStr">
         <is>
-          <t>Sep-26</t>
+          <t>Oct-26</t>
         </is>
       </c>
       <c r="D483" s="2" t="n">
-        <v>46266</v>
+        <v>46296</v>
       </c>
       <c r="E483" t="inlineStr">
         <is>
@@ -22535,7 +22535,7 @@
       </c>
       <c r="F483" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>High</t>
         </is>
       </c>
     </row>
@@ -22552,11 +22552,11 @@
       </c>
       <c r="C484" t="inlineStr">
         <is>
-          <t>Oct-26</t>
+          <t>Nov-26</t>
         </is>
       </c>
       <c r="D484" s="2" t="n">
-        <v>46296</v>
+        <v>46327</v>
       </c>
       <c r="E484" t="inlineStr">
         <is>
@@ -22565,7 +22565,7 @@
       </c>
       <c r="F484" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>High</t>
         </is>
       </c>
     </row>

</xml_diff>